<commit_message>
chore: migrate GSC token to public directory for Vite compilation asset passing
</commit_message>
<xml_diff>
--- a/Baking_calculator project log.xlsx
+++ b/Baking_calculator project log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\James\OneDrive\Documents\1_AppDesignStudio_work\2_WEB_DEV\1_Production\1. App_Design_Studio_Products_Live\baking-hydration-calculator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F018900-602B-4EF1-9CE7-DD836AAC72CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D1D3787-4F5D-419B-B731-307A67B58949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-1200" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Task_Log" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="SRS_freeze_notice" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="93">
   <si>
     <t>Task ID</t>
   </si>
@@ -434,6 +435,15 @@
   </si>
   <si>
     <t>In Progress</t>
+  </si>
+  <si>
+    <t>Environment Consolidation – Remove custom domain association from the duplicate manual project sensational-jalebi-dcf6d5, decommission the duplicate instance, and bind the active baking.headsup-consulting.com subdomain to your clean, GitHub-linked baking-hydration-calculator project.</t>
+  </si>
+  <si>
+    <t>Execute Project Phase: CI/CD Pipeline Integration – Decommission the legacy manual deployment of spacing-calculator, establish the GitHub-to-Netlify build pipeline for jamespnz/spacing-calculator, and assign spacing.headsup-consulting.com as the primary secure production domain.</t>
+  </si>
+  <si>
+    <t>Update the configuration management baseline by saving the high-trust strategic instructions to the user profile memory, officially incorporating the new operational principles into the system development life cycle. Language Style: PMI PMBOK Guide 7th Edition metrics.</t>
   </si>
 </sst>
 </file>
@@ -504,7 +514,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -526,6 +536,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -572,7 +594,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -621,6 +643,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -934,15 +962,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultColWidth="63.140625" defaultRowHeight="38.25" customHeight="1"/>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultColWidth="63.109375" defaultRowHeight="38.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" customWidth="1"/>
-    <col min="4" max="4" width="26.28515625" customWidth="1"/>
-    <col min="5" max="5" width="25.140625" customWidth="1"/>
-    <col min="6" max="6" width="21.5703125" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.88671875" customWidth="1"/>
+    <col min="3" max="3" width="80.44140625" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" customWidth="1"/>
+    <col min="5" max="5" width="25.109375" customWidth="1"/>
+    <col min="6" max="6" width="21.5546875" customWidth="1"/>
+    <col min="7" max="7" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="38.25" customHeight="1" thickBot="1">
@@ -978,7 +1007,7 @@
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="18" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1115,55 +1144,93 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" ht="38.25" customHeight="1" thickBot="1">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:8" ht="60" customHeight="1" thickBot="1">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="60" customHeight="1" thickBot="1">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="60" customHeight="1" thickBot="1">
+      <c r="A10" s="1"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" ht="38.25" customHeight="1" thickBot="1">
+      <c r="A11" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="38.25" customHeight="1" thickBot="1">
-      <c r="A9" s="1" t="s">
+    <row r="12" spans="1:8" ht="38.25" customHeight="1" thickBot="1">
+      <c r="A12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1186,9 +1253,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E1614D7-DFB7-43C1-BCFF-6B6906ED5C1F}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="27.42578125" customWidth="1"/>
+    <col min="1" max="1" width="27.44140625" customWidth="1"/>
     <col min="2" max="2" width="57" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1279,10 +1346,10 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="50" defaultRowHeight="27.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" customWidth="1"/>
-    <col min="3" max="3" width="42.28515625" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" customWidth="1"/>
+    <col min="3" max="3" width="42.33203125" customWidth="1"/>
+    <col min="4" max="4" width="23.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.75" customHeight="1" thickBot="1">
@@ -1321,12 +1388,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{676866DD-4272-4736-860C-06096EEFBD27}">
   <dimension ref="A1:A33"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="189.85546875" customWidth="1"/>
+    <col min="1" max="1" width="189.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="23.25">
+    <row r="1" spans="1:1" ht="22.8">
       <c r="A1" s="9" t="s">
         <v>51</v>
       </c>
@@ -1351,7 +1418,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="23.25">
+    <row r="6" spans="1:1" ht="22.8">
       <c r="A6" s="9" t="s">
         <v>56</v>
       </c>
@@ -1371,7 +1438,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="23.25">
+    <row r="10" spans="1:1" ht="22.8">
       <c r="A10" s="9" t="s">
         <v>60</v>
       </c>
@@ -1381,7 +1448,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="17.25">
+    <row r="12" spans="1:1" ht="17.399999999999999">
       <c r="A12" s="13" t="s">
         <v>62</v>
       </c>
@@ -1411,7 +1478,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="17.25">
+    <row r="18" spans="1:1" ht="17.399999999999999">
       <c r="A18" s="13" t="s">
         <v>68</v>
       </c>
@@ -1426,7 +1493,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="17.25">
+    <row r="21" spans="1:1" ht="17.399999999999999">
       <c r="A21" s="13" t="s">
         <v>71</v>
       </c>
@@ -1436,7 +1503,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="15.75">
+    <row r="23" spans="1:1" ht="15.6">
       <c r="A23" s="15" t="s">
         <v>73</v>
       </c>
@@ -1451,7 +1518,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="15.75">
+    <row r="26" spans="1:1" ht="15.6">
       <c r="A26" s="15" t="s">
         <v>76</v>
       </c>
@@ -1471,10 +1538,10 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="23.25">
+    <row r="30" spans="1:1" ht="22.8">
       <c r="A30" s="9"/>
     </row>
-    <row r="31" spans="1:1" ht="17.25">
+    <row r="31" spans="1:1" ht="17.399999999999999">
       <c r="A31" s="13"/>
     </row>
     <row r="32" spans="1:1">

</xml_diff>